<commit_message>
chore(release): bump version to v1.1.21, sync updated pricelist, and add langganan checklist to publisher input
</commit_message>
<xml_diff>
--- a/Harga Percetakan (2).xlsx
+++ b/Harga Percetakan (2).xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Harga Normal" sheetId="1" state="visible" r:id="rId1"/>
@@ -169,18 +169,21 @@
     <t>Keterangan</t>
   </si>
   <si>
+    <t xml:space="preserve">diskon 10%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cover cetak Offset + minimal 200 hal</t>
+  </si>
+  <si>
     <t xml:space="preserve">diskon 25%</t>
   </si>
   <si>
-    <t xml:space="preserve">Cover cetak Offset + minimal 200 hal</t>
+    <t>1000-2500</t>
   </si>
   <si>
     <t xml:space="preserve">diskon 50%</t>
   </si>
   <si>
-    <t xml:space="preserve">diskon 80%</t>
-  </si>
-  <si>
     <t xml:space="preserve">Harga Laminasi</t>
   </si>
   <si>
@@ -245,9 +248,6 @@
   </si>
   <si>
     <t>A4/B5</t>
-  </si>
-  <si>
-    <t>1000-2500</t>
   </si>
   <si>
     <t xml:space="preserve">diskon 75%</t>
@@ -402,7 +402,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="164" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -464,7 +464,12 @@
     <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="4" numFmtId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="4" numFmtId="165" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf fontId="2" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1446,11 +1451,11 @@
       <c r="G31" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="H31" s="26" t="s">
+      <c r="H31" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="I31" s="26"/>
-      <c r="J31" s="26"/>
+      <c r="I31" s="27"/>
+      <c r="J31" s="27"/>
     </row>
     <row r="32">
       <c r="B32" s="7" t="s">
@@ -1468,11 +1473,11 @@
       <c r="G32" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="H32" s="26" t="s">
+      <c r="H32" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="I32" s="26"/>
-      <c r="J32" s="26"/>
+      <c r="I32" s="27"/>
+      <c r="J32" s="27"/>
     </row>
     <row r="33">
       <c r="B33" s="7" t="s">
@@ -1484,17 +1489,17 @@
       <c r="D33" s="9">
         <v>12750</v>
       </c>
-      <c r="F33" s="27">
-        <v>1000</v>
+      <c r="F33" s="28" t="s">
+        <v>53</v>
       </c>
       <c r="G33" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="H33" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="H33" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="I33" s="26"/>
-      <c r="J33" s="26"/>
+      <c r="I33" s="27"/>
+      <c r="J33" s="27"/>
     </row>
     <row r="34">
       <c r="B34" s="7" t="s">
@@ -1509,186 +1514,186 @@
     </row>
     <row r="37">
       <c r="B37" s="15" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="C38" s="28">
+        <v>56</v>
+      </c>
+      <c r="C38" s="29">
         <v>1500</v>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="C41" s="28">
+        <v>58</v>
+      </c>
+      <c r="C41" s="29">
         <v>5000</v>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="15" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="29" t="s">
+      <c r="B44" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="C44" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="D44" s="29" t="s">
+      <c r="C44" s="30" t="s">
         <v>60</v>
       </c>
+      <c r="D44" s="30" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="45">
-      <c r="B45" s="26" t="s">
-        <v>61</v>
-      </c>
-      <c r="C45" s="30">
+      <c r="B45" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="C45" s="31">
         <v>500</v>
       </c>
-      <c r="D45" s="31">
+      <c r="D45" s="32">
         <v>600</v>
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="C46" s="30">
+      <c r="B46" s="27" t="s">
+        <v>63</v>
+      </c>
+      <c r="C46" s="31">
         <v>550</v>
       </c>
-      <c r="D46" s="31">
+      <c r="D46" s="32">
         <v>650</v>
       </c>
     </row>
     <row r="47">
-      <c r="B47" s="26" t="s">
-        <v>63</v>
-      </c>
-      <c r="C47" s="30">
+      <c r="B47" s="27" t="s">
+        <v>64</v>
+      </c>
+      <c r="C47" s="31">
         <v>600</v>
       </c>
-      <c r="D47" s="31">
+      <c r="D47" s="32">
         <v>700</v>
       </c>
     </row>
     <row r="48">
-      <c r="B48" s="26" t="s">
-        <v>64</v>
-      </c>
-      <c r="C48" s="30">
+      <c r="B48" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="C48" s="31">
         <v>650</v>
       </c>
-      <c r="D48" s="31">
+      <c r="D48" s="32">
         <v>750</v>
       </c>
     </row>
     <row r="49">
-      <c r="B49" s="26" t="s">
-        <v>65</v>
-      </c>
-      <c r="C49" s="30">
+      <c r="B49" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="C49" s="31">
         <v>700</v>
       </c>
-      <c r="D49" s="31">
+      <c r="D49" s="32">
         <v>800</v>
       </c>
     </row>
     <row r="50">
-      <c r="B50" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="C50" s="30">
+      <c r="B50" s="27" t="s">
+        <v>67</v>
+      </c>
+      <c r="C50" s="31">
         <v>750</v>
       </c>
-      <c r="D50" s="31">
+      <c r="D50" s="32">
         <v>850</v>
       </c>
     </row>
     <row r="51">
-      <c r="B51" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="C51" s="30">
+      <c r="B51" s="27" t="s">
+        <v>68</v>
+      </c>
+      <c r="C51" s="31">
         <v>800</v>
       </c>
-      <c r="D51" s="31">
+      <c r="D51" s="32">
         <v>950</v>
       </c>
     </row>
     <row r="52">
-      <c r="B52" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="C52" s="30">
+      <c r="B52" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="C52" s="31">
         <v>850</v>
       </c>
-      <c r="D52" s="31">
+      <c r="D52" s="32">
         <v>1150</v>
       </c>
     </row>
     <row r="53">
-      <c r="B53" s="26" t="s">
-        <v>69</v>
-      </c>
-      <c r="C53" s="30">
+      <c r="B53" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="C53" s="31">
         <v>900</v>
       </c>
-      <c r="D53" s="31">
+      <c r="D53" s="32">
         <v>1250</v>
       </c>
     </row>
     <row r="54">
-      <c r="B54" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="C54" s="30">
+      <c r="B54" s="27" t="s">
+        <v>71</v>
+      </c>
+      <c r="C54" s="31">
         <v>950</v>
       </c>
-      <c r="D54" s="31">
+      <c r="D54" s="32">
         <v>1350</v>
       </c>
     </row>
     <row r="55">
-      <c r="B55" s="26" t="s">
-        <v>71</v>
-      </c>
-      <c r="C55" s="30">
+      <c r="B55" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="C55" s="31">
         <v>1000</v>
       </c>
-      <c r="D55" s="31">
+      <c r="D55" s="32">
         <v>1550</v>
       </c>
     </row>
     <row r="56">
-      <c r="B56" s="26" t="s">
-        <v>72</v>
-      </c>
-      <c r="C56" s="30">
+      <c r="B56" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="C56" s="31">
         <v>1050</v>
       </c>
-      <c r="D56" s="31">
+      <c r="D56" s="32">
         <v>1750</v>
       </c>
     </row>
     <row r="57">
-      <c r="B57" s="26" t="s">
-        <v>73</v>
-      </c>
-      <c r="C57" s="30">
+      <c r="B57" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="C57" s="31">
         <v>1100</v>
       </c>
-      <c r="D57" s="31">
+      <c r="D57" s="32">
         <v>1950</v>
       </c>
     </row>
@@ -1974,7 +1979,7 @@
         <v>5000</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G20" s="8" t="s">
         <v>29</v>
@@ -1994,7 +1999,7 @@
         <v>5500</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G21" s="8" t="s">
         <v>29</v>
@@ -2144,14 +2149,14 @@
       <c r="F31" s="8">
         <v>300</v>
       </c>
-      <c r="G31" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="H31" s="26" t="s">
+      <c r="G31" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="H31" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="I31" s="26"/>
-      <c r="J31" s="26"/>
+      <c r="I31" s="27"/>
+      <c r="J31" s="27"/>
     </row>
     <row r="32">
       <c r="B32" s="7" t="s">
@@ -2166,14 +2171,14 @@
       <c r="F32" s="8">
         <v>500</v>
       </c>
-      <c r="G32" s="26" t="s">
-        <v>52</v>
-      </c>
-      <c r="H32" s="26" t="s">
+      <c r="G32" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="H32" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="I32" s="26"/>
-      <c r="J32" s="26"/>
+      <c r="I32" s="27"/>
+      <c r="J32" s="27"/>
     </row>
     <row r="33">
       <c r="B33" s="7" t="s">
@@ -2185,17 +2190,17 @@
       <c r="D33" s="9">
         <v>11000</v>
       </c>
-      <c r="F33" s="32" t="s">
-        <v>76</v>
-      </c>
-      <c r="G33" s="26" t="s">
+      <c r="F33" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="G33" s="27" t="s">
         <v>77</v>
       </c>
-      <c r="H33" s="26" t="s">
+      <c r="H33" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="I33" s="26"/>
-      <c r="J33" s="26"/>
+      <c r="I33" s="27"/>
+      <c r="J33" s="27"/>
     </row>
     <row r="34">
       <c r="B34" s="7" t="s">
@@ -2210,186 +2215,186 @@
     </row>
     <row r="37">
       <c r="B37" s="15" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="C38" s="28">
+        <v>56</v>
+      </c>
+      <c r="C38" s="29">
         <v>1000</v>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="C41" s="28">
+        <v>58</v>
+      </c>
+      <c r="C41" s="29">
         <v>3000</v>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="15" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="29" t="s">
+      <c r="B44" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="C44" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="D44" s="29" t="s">
+      <c r="C44" s="30" t="s">
         <v>60</v>
       </c>
+      <c r="D44" s="30" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="45">
-      <c r="B45" s="26" t="s">
-        <v>61</v>
-      </c>
-      <c r="C45" s="30">
+      <c r="B45" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="C45" s="31">
         <v>500</v>
       </c>
-      <c r="D45" s="31">
+      <c r="D45" s="32">
         <v>600</v>
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="C46" s="30">
+      <c r="B46" s="27" t="s">
+        <v>63</v>
+      </c>
+      <c r="C46" s="31">
         <v>550</v>
       </c>
-      <c r="D46" s="31">
+      <c r="D46" s="32">
         <v>650</v>
       </c>
     </row>
     <row r="47">
-      <c r="B47" s="26" t="s">
-        <v>63</v>
-      </c>
-      <c r="C47" s="30">
+      <c r="B47" s="27" t="s">
+        <v>64</v>
+      </c>
+      <c r="C47" s="31">
         <v>600</v>
       </c>
-      <c r="D47" s="31">
+      <c r="D47" s="32">
         <v>700</v>
       </c>
     </row>
     <row r="48">
-      <c r="B48" s="26" t="s">
-        <v>64</v>
-      </c>
-      <c r="C48" s="30">
+      <c r="B48" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="C48" s="31">
         <v>650</v>
       </c>
-      <c r="D48" s="31">
+      <c r="D48" s="32">
         <v>750</v>
       </c>
     </row>
     <row r="49">
-      <c r="B49" s="26" t="s">
-        <v>65</v>
-      </c>
-      <c r="C49" s="30">
+      <c r="B49" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="C49" s="31">
         <v>700</v>
       </c>
-      <c r="D49" s="31">
+      <c r="D49" s="32">
         <v>800</v>
       </c>
     </row>
     <row r="50">
-      <c r="B50" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="C50" s="30">
+      <c r="B50" s="27" t="s">
+        <v>67</v>
+      </c>
+      <c r="C50" s="31">
         <v>750</v>
       </c>
-      <c r="D50" s="31">
+      <c r="D50" s="32">
         <v>850</v>
       </c>
     </row>
     <row r="51">
-      <c r="B51" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="C51" s="30">
+      <c r="B51" s="27" t="s">
+        <v>68</v>
+      </c>
+      <c r="C51" s="31">
         <v>800</v>
       </c>
-      <c r="D51" s="31">
+      <c r="D51" s="32">
         <v>950</v>
       </c>
     </row>
     <row r="52">
-      <c r="B52" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="C52" s="30">
+      <c r="B52" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="C52" s="31">
         <v>850</v>
       </c>
-      <c r="D52" s="31">
+      <c r="D52" s="32">
         <v>1150</v>
       </c>
     </row>
     <row r="53">
-      <c r="B53" s="26" t="s">
-        <v>69</v>
-      </c>
-      <c r="C53" s="30">
+      <c r="B53" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="C53" s="31">
         <v>900</v>
       </c>
-      <c r="D53" s="31">
+      <c r="D53" s="32">
         <v>1250</v>
       </c>
     </row>
     <row r="54">
-      <c r="B54" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="C54" s="30">
+      <c r="B54" s="27" t="s">
+        <v>71</v>
+      </c>
+      <c r="C54" s="31">
         <v>950</v>
       </c>
-      <c r="D54" s="31">
+      <c r="D54" s="32">
         <v>1350</v>
       </c>
     </row>
     <row r="55">
-      <c r="B55" s="26" t="s">
-        <v>71</v>
-      </c>
-      <c r="C55" s="30">
+      <c r="B55" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="C55" s="31">
         <v>1000</v>
       </c>
-      <c r="D55" s="31">
+      <c r="D55" s="32">
         <v>1550</v>
       </c>
     </row>
     <row r="56">
-      <c r="B56" s="26" t="s">
-        <v>72</v>
-      </c>
-      <c r="C56" s="30">
+      <c r="B56" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="C56" s="31">
         <v>1050</v>
       </c>
-      <c r="D56" s="31">
+      <c r="D56" s="32">
         <v>1750</v>
       </c>
     </row>
     <row r="57">
-      <c r="B57" s="26" t="s">
-        <v>73</v>
-      </c>
-      <c r="C57" s="30">
+      <c r="B57" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="C57" s="31">
         <v>1100</v>
       </c>
-      <c r="D57" s="31">
+      <c r="D57" s="32">
         <v>1950</v>
       </c>
     </row>

</xml_diff>